<commit_message>
Catat konfirmasi petugas, izin data, dan batas data Okt 2026
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sigizi/analisis/Analisis_Stunting_Mumbulsari.xlsx
+++ b/data/sigizi/analisis/Analisis_Stunting_Mumbulsari.xlsx
@@ -2623,7 +2623,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mini Riset KOAS IKM, FK Universitas Jember · data SigiziKesga (sigizikesga.kemkes.go.id) · Jan 2024–Sep 2026 · 7 desa · 108.322 pengukuran, 6.312 anak · diolah 19 Okt 2026</t>
+          <t>Mini Riset KOAS IKM, FK Universitas Jember · data SigiziKesga (sigizikesga.kemkes.go.id) · Jan 2024–Sep 2026 · 7 desa · 108.322 pengukuran, 6.312 anak · data diambil 19 Okt 2026; Okt 2026 tidak dianalisis (baru 20 pengukuran, sampai 19 Okt)</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
     <row r="31" ht="50" customHeight="1">
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Data ini adalah data rutin (entri petugas) dengan masalah kualitas yang terdokumentasi (sheet 12). Semua hasil adalah asosiasi pada data observasional. Verifikasi dengan petugas entri Puskesmas dan izin penggunaan data tetap perlu dikonfirmasi sebelum publikasi. Tidak ada data pribadi di berkas ini.</t>
+          <t>Data ini adalah data rutin (entri petugas) dengan masalah kualitas yang terdokumentasi (sheet 12). Semua hasil adalah asosiasi pada data observasional. Petugas entri Puskesmas telah mengonfirmasi (20 Okt 2026) bahwa sebagian desa mengisi satu tanggal ukur per bulan dan tinggi badan dibulatkan. Izin penggunaan data ada dan dilampirkan terpisah. Tidak ada data pribadi di berkas ini.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pindahkan analisis ke SPSS dan R, laporan dan workbook membaca hasil barunya
- SPSS 27 (skrip/spss): a3, a4, a5 uji, p2; dijalankan tanpa antarmuka lewat jalankan_spss.py
- R (analisis_r_1..3.R): a1, a2, a5 tabel, a6-a9, p1, p3; cleaning dan skenario tetap di Python
- siapkan_data_spss_r.py meneruskan sampel acak per anak per tahun dari Python agar uji sama persis
- bandingkan_hasil.R: semua kolom deterministik sama dengan Python; hanya batas CI bootstrap dan simulasi bergeser
- gabung_hasil_rs.py membentuk data/sigizi/analisis_rs untuk laporan dan workbook
- Workbook dan tabel laporan dibangun ulang; teks Bab 3 dan IK stunting S0 (Bab 4.2) disesuaikan
- .docx belum dibangun ulang (lihat data/sigizi/laporan/README.md)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sigizi/analisis/Analisis_Stunting_Mumbulsari.xlsx
+++ b/data/sigizi/analisis/Analisis_Stunting_Mumbulsari.xlsx
@@ -55033,7 +55033,7 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>6.0–7.0</t>
+          <t>6.0–7.1</t>
         </is>
       </c>
       <c r="D6" s="14" t="n">
@@ -55049,7 +55049,7 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>6.5–7.6</t>
+          <t>6.4–7.6</t>
         </is>
       </c>
       <c r="H6" s="14" t="n">
@@ -55057,7 +55057,7 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>5.7–6.7</t>
+          <t>5.7–6.8</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
@@ -55088,7 +55088,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>5.7–9.3</t>
+          <t>5.8–9.5</t>
         </is>
       </c>
       <c r="D7" s="16" t="n">
@@ -55096,7 +55096,7 @@
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>9.3–13.2</t>
+          <t>9.2–13.3</t>
         </is>
       </c>
       <c r="F7" s="16" t="n">
@@ -55104,7 +55104,7 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>6.1–9.0</t>
+          <t>6.2–9.1</t>
         </is>
       </c>
       <c r="H7" s="16" t="n">
@@ -55112,7 +55112,7 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>5.9–9.7</t>
+          <t>5.7–9.2</t>
         </is>
       </c>
       <c r="J7" s="16" t="n">
@@ -55120,7 +55120,7 @@
       </c>
       <c r="K7" s="15" t="inlineStr">
         <is>
-          <t>9.3–13.4</t>
+          <t>9.0–13.3</t>
         </is>
       </c>
       <c r="L7" s="16" t="n">
@@ -55128,7 +55128,7 @@
       </c>
       <c r="M7" s="15" t="inlineStr">
         <is>
-          <t>6.1–9.1</t>
+          <t>5.9–9.0</t>
         </is>
       </c>
     </row>
@@ -55151,7 +55151,7 @@
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>4.8–9.0</t>
+          <t>4.7–8.9</t>
         </is>
       </c>
       <c r="F8" s="14" t="n">
@@ -55159,7 +55159,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>6.6–11.8</t>
+          <t>6.4–12.0</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
@@ -55167,7 +55167,7 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>5.5–9.0</t>
+          <t>5.4–9.1</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
@@ -55175,7 +55175,7 @@
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>4.9–9.0</t>
+          <t>4.6–9.2</t>
         </is>
       </c>
       <c r="L8" s="14" t="n">
@@ -55183,7 +55183,7 @@
       </c>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>6.5–11.4</t>
+          <t>6.7–11.9</t>
         </is>
       </c>
     </row>
@@ -55206,7 +55206,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>4.8–7.6</t>
+          <t>4.9–7.6</t>
         </is>
       </c>
       <c r="F9" s="16" t="n">
@@ -55214,7 +55214,7 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>1.1–1.7</t>
+          <t>1.1–1.8</t>
         </is>
       </c>
       <c r="H9" s="16" t="n">
@@ -55222,7 +55222,7 @@
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>3.9–5.6</t>
+          <t>3.9–5.7</t>
         </is>
       </c>
       <c r="J9" s="16" t="n">
@@ -55230,7 +55230,7 @@
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>4.9–7.7</t>
+          <t>4.9–7.6</t>
         </is>
       </c>
       <c r="L9" s="16" t="n">
@@ -55253,7 +55253,7 @@
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>12.3–15.6</t>
+          <t>12.5–15.4</t>
         </is>
       </c>
       <c r="D10" s="14" t="n">
@@ -55261,7 +55261,7 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>21.2–27.6</t>
+          <t>20.9–27.4</t>
         </is>
       </c>
       <c r="F10" s="14" t="n">
@@ -55277,7 +55277,7 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>9.5–12.6</t>
+          <t>9.6–12.5</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
@@ -55285,7 +55285,7 @@
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>25.6–33.5</t>
+          <t>25.6–33.3</t>
         </is>
       </c>
       <c r="L10" s="14" t="n">
@@ -55308,7 +55308,7 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>3.2–5.2</t>
+          <t>3.1–5.1</t>
         </is>
       </c>
       <c r="D11" s="16" t="n">
@@ -55316,7 +55316,7 @@
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>26.1–30.4</t>
+          <t>26.3–30.8</t>
         </is>
       </c>
       <c r="F11" s="16" t="n">
@@ -55324,7 +55324,7 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>1.4–2.3</t>
+          <t>1.5–2.4</t>
         </is>
       </c>
       <c r="H11" s="16" t="n">
@@ -55332,7 +55332,7 @@
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>3.4–5.0</t>
+          <t>3.3–5.2</t>
         </is>
       </c>
       <c r="J11" s="16" t="n">
@@ -55340,7 +55340,7 @@
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>27.0–31.9</t>
+          <t>27.2–31.7</t>
         </is>
       </c>
       <c r="L11" s="16" t="n">
@@ -55348,7 +55348,7 @@
       </c>
       <c r="M11" s="15" t="inlineStr">
         <is>
-          <t>0.6–1.1</t>
+          <t>0.5–1.1</t>
         </is>
       </c>
     </row>
@@ -55363,7 +55363,7 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>7.4–10.2</t>
+          <t>7.4–10.1</t>
         </is>
       </c>
       <c r="D12" s="14" t="n">
@@ -55371,7 +55371,7 @@
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>6.8–10.3</t>
+          <t>7.0–10.2</t>
         </is>
       </c>
       <c r="F12" s="14" t="n">
@@ -55379,7 +55379,7 @@
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>18.8–24.0</t>
+          <t>19.0–24.6</t>
         </is>
       </c>
       <c r="H12" s="14" t="n">
@@ -55387,7 +55387,7 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>7.2–10.2</t>
+          <t>7.3–10.5</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
@@ -55395,7 +55395,7 @@
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>6.8–10.1</t>
+          <t>6.9–10.0</t>
         </is>
       </c>
       <c r="L12" s="14" t="n">
@@ -55403,7 +55403,7 @@
       </c>
       <c r="M12" s="13" t="inlineStr">
         <is>
-          <t>19.1–24.5</t>
+          <t>19.0–24.1</t>
         </is>
       </c>
     </row>
@@ -55426,7 +55426,7 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>12.2–17.3</t>
+          <t>12.3–17.6</t>
         </is>
       </c>
       <c r="F13" s="16" t="n">
@@ -55434,7 +55434,7 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>7.2–10.5</t>
+          <t>7.3–10.5</t>
         </is>
       </c>
       <c r="H13" s="16" t="n">
@@ -55442,7 +55442,7 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>0.4–2.5</t>
+          <t>0.4–2.3</t>
         </is>
       </c>
       <c r="J13" s="16" t="n">
@@ -55450,7 +55450,7 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>11.5–16.7</t>
+          <t>11.4–16.5</t>
         </is>
       </c>
       <c r="L13" s="16" t="n">
@@ -55458,7 +55458,7 @@
       </c>
       <c r="M13" s="15" t="inlineStr">
         <is>
-          <t>7.8–11.4</t>
+          <t>8.0–11.5</t>
         </is>
       </c>
     </row>
@@ -55547,7 +55547,7 @@
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>7.1–8.3</t>
+          <t>7.1–8.4</t>
         </is>
       </c>
       <c r="D17" s="14" t="n">
@@ -55563,7 +55563,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>5.6–6.5</t>
+          <t>5.6–6.6</t>
         </is>
       </c>
       <c r="H17" s="14" t="n">
@@ -55571,7 +55571,7 @@
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>7.1–8.4</t>
+          <t>7.1–8.3</t>
         </is>
       </c>
       <c r="J17" s="14" t="n">
@@ -55602,7 +55602,7 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>8.7–12.7</t>
+          <t>8.5–12.4</t>
         </is>
       </c>
       <c r="D18" s="16" t="n">
@@ -55610,7 +55610,7 @@
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>5.8–9.4</t>
+          <t>6.0–9.3</t>
         </is>
       </c>
       <c r="F18" s="16" t="n">
@@ -55618,7 +55618,7 @@
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>7.8–11.1</t>
+          <t>8.0–11.1</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
@@ -55626,7 +55626,7 @@
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>8.5–12.5</t>
+          <t>8.7–12.5</t>
         </is>
       </c>
       <c r="J18" s="16" t="n">
@@ -55634,7 +55634,7 @@
       </c>
       <c r="K18" s="15" t="inlineStr">
         <is>
-          <t>5.9–9.5</t>
+          <t>5.7–9.4</t>
         </is>
       </c>
       <c r="L18" s="16" t="n">
@@ -55642,7 +55642,7 @@
       </c>
       <c r="M18" s="15" t="inlineStr">
         <is>
-          <t>7.8–11.3</t>
+          <t>7.7–11.5</t>
         </is>
       </c>
     </row>
@@ -55657,7 +55657,7 @@
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>10.1–14.7</t>
+          <t>10.0–15.1</t>
         </is>
       </c>
       <c r="D19" s="14" t="n">
@@ -55665,7 +55665,7 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>3.6–6.7</t>
+          <t>3.6–6.6</t>
         </is>
       </c>
       <c r="F19" s="14" t="n">
@@ -55673,7 +55673,7 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>4.6–8.3</t>
+          <t>4.7–8.3</t>
         </is>
       </c>
       <c r="H19" s="14" t="n">
@@ -55681,7 +55681,7 @@
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>9.9–14.9</t>
+          <t>10.1–15.1</t>
         </is>
       </c>
       <c r="J19" s="14" t="n">
@@ -55689,7 +55689,7 @@
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>3.5–6.8</t>
+          <t>3.6–6.6</t>
         </is>
       </c>
       <c r="L19" s="14" t="n">
@@ -55697,7 +55697,7 @@
       </c>
       <c r="M19" s="13" t="inlineStr">
         <is>
-          <t>4.6–8.2</t>
+          <t>4.5–8.4</t>
         </is>
       </c>
     </row>
@@ -55712,7 +55712,7 @@
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>1.0–1.9</t>
+          <t>1.1–1.9</t>
         </is>
       </c>
       <c r="D20" s="16" t="n">
@@ -55720,7 +55720,7 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>2.8–4.5</t>
+          <t>2.9–4.4</t>
         </is>
       </c>
       <c r="F20" s="16" t="n">
@@ -55736,7 +55736,7 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>1.1–1.9</t>
+          <t>1.0–1.9</t>
         </is>
       </c>
       <c r="J20" s="16" t="n">
@@ -55767,7 +55767,7 @@
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>3.1–4.8</t>
+          <t>3.1–5.0</t>
         </is>
       </c>
       <c r="D21" s="14" t="n">
@@ -55775,7 +55775,7 @@
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>3.1–5.2</t>
+          <t>3.1–5.1</t>
         </is>
       </c>
       <c r="F21" s="14" t="n">
@@ -55791,7 +55791,7 @@
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>2.4–4.1</t>
+          <t>2.5–4.1</t>
         </is>
       </c>
       <c r="J21" s="14" t="n">
@@ -55799,7 +55799,7 @@
       </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
-          <t>1.5–3.6</t>
+          <t>1.4–3.6</t>
         </is>
       </c>
       <c r="L21" s="14" t="n">
@@ -55807,7 +55807,7 @@
       </c>
       <c r="M21" s="13" t="inlineStr">
         <is>
-          <t>1.7–2.7</t>
+          <t>1.6–2.8</t>
         </is>
       </c>
     </row>
@@ -55822,7 +55822,7 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>0.7–1.7</t>
+          <t>0.8–1.7</t>
         </is>
       </c>
       <c r="D22" s="16" t="n">
@@ -55830,7 +55830,7 @@
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>7.5–9.8</t>
+          <t>7.4–9.8</t>
         </is>
       </c>
       <c r="F22" s="16" t="n">
@@ -55838,7 +55838,7 @@
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>3.3–4.2</t>
+          <t>3.2–4.1</t>
         </is>
       </c>
       <c r="H22" s="16" t="n">
@@ -55846,7 +55846,7 @@
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>0.7–1.7</t>
+          <t>0.7–1.8</t>
         </is>
       </c>
       <c r="J22" s="16" t="n">
@@ -55854,7 +55854,7 @@
       </c>
       <c r="K22" s="15" t="inlineStr">
         <is>
-          <t>7.8–10.2</t>
+          <t>7.8–10.1</t>
         </is>
       </c>
       <c r="L22" s="16" t="n">
@@ -55862,7 +55862,7 @@
       </c>
       <c r="M22" s="15" t="inlineStr">
         <is>
-          <t>4.5–5.8</t>
+          <t>4.5–5.7</t>
         </is>
       </c>
     </row>
@@ -55877,7 +55877,7 @@
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>20.1–24.6</t>
+          <t>20.1–24.5</t>
         </is>
       </c>
       <c r="D23" s="14" t="n">
@@ -55885,7 +55885,7 @@
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>18.6–23.1</t>
+          <t>18.3–22.9</t>
         </is>
       </c>
       <c r="F23" s="14" t="n">
@@ -55893,7 +55893,7 @@
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>14.5–19.0</t>
+          <t>14.7–18.6</t>
         </is>
       </c>
       <c r="H23" s="14" t="n">
@@ -55901,7 +55901,7 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>20.0–24.8</t>
+          <t>20.2–24.5</t>
         </is>
       </c>
       <c r="J23" s="14" t="n">
@@ -55909,7 +55909,7 @@
       </c>
       <c r="K23" s="13" t="inlineStr">
         <is>
-          <t>18.3–22.7</t>
+          <t>18.4–23.0</t>
         </is>
       </c>
       <c r="L23" s="14" t="n">
@@ -55917,7 +55917,7 @@
       </c>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>14.4–18.9</t>
+          <t>14.3–18.8</t>
         </is>
       </c>
     </row>
@@ -55932,7 +55932,7 @@
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>0.9–1.9</t>
+          <t>1.0–2.0</t>
         </is>
       </c>
       <c r="D24" s="16" t="n">
@@ -55940,7 +55940,7 @@
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>5.0–8.6</t>
+          <t>5.2–8.7</t>
         </is>
       </c>
       <c r="F24" s="16" t="n">
@@ -55948,7 +55948,7 @@
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>5.5–8.2</t>
+          <t>5.4–8.2</t>
         </is>
       </c>
       <c r="H24" s="16" t="n">
@@ -55956,7 +55956,7 @@
       </c>
       <c r="I24" s="15" t="inlineStr">
         <is>
-          <t>0.9–1.9</t>
+          <t>1.0–1.9</t>
         </is>
       </c>
       <c r="J24" s="16" t="n">
@@ -55964,7 +55964,7 @@
       </c>
       <c r="K24" s="15" t="inlineStr">
         <is>
-          <t>5.0–8.6</t>
+          <t>4.7–8.4</t>
         </is>
       </c>
       <c r="L24" s="16" t="n">
@@ -55972,7 +55972,7 @@
       </c>
       <c r="M24" s="15" t="inlineStr">
         <is>
-          <t>4.7–7.4</t>
+          <t>4.6–7.3</t>
         </is>
       </c>
     </row>
@@ -56077,7 +56077,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>10.0–11.2</t>
+          <t>10.0–11.3</t>
         </is>
       </c>
       <c r="H28" s="14" t="n">
@@ -56085,7 +56085,7 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>9.1–10.7</t>
+          <t>9.1–10.6</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
@@ -56093,7 +56093,7 @@
       </c>
       <c r="K28" s="13" t="inlineStr">
         <is>
-          <t>11.8–13.7</t>
+          <t>11.9–13.6</t>
         </is>
       </c>
       <c r="L28" s="14" t="n">
@@ -56116,7 +56116,7 @@
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>12.9–18.6</t>
+          <t>12.7–18.4</t>
         </is>
       </c>
       <c r="D29" s="16" t="n">
@@ -56124,7 +56124,7 @@
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>12.3–17.4</t>
+          <t>12.2–17.7</t>
         </is>
       </c>
       <c r="F29" s="16" t="n">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="G29" s="15" t="inlineStr">
         <is>
-          <t>12.8–17.0</t>
+          <t>12.8–17.2</t>
         </is>
       </c>
       <c r="H29" s="16" t="n">
@@ -56140,7 +56140,7 @@
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>12.7–18.6</t>
+          <t>12.8–18.4</t>
         </is>
       </c>
       <c r="J29" s="16" t="n">
@@ -56148,7 +56148,7 @@
       </c>
       <c r="K29" s="15" t="inlineStr">
         <is>
-          <t>12.4–17.5</t>
+          <t>12.4–18.0</t>
         </is>
       </c>
       <c r="L29" s="16" t="n">
@@ -56156,7 +56156,7 @@
       </c>
       <c r="M29" s="15" t="inlineStr">
         <is>
-          <t>12.5–17.2</t>
+          <t>12.6–17.0</t>
         </is>
       </c>
     </row>
@@ -56171,7 +56171,7 @@
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>14.6–21.2</t>
+          <t>14.5–21.3</t>
         </is>
       </c>
       <c r="D30" s="14" t="n">
@@ -56179,7 +56179,7 @@
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>6.7–11.4</t>
+          <t>6.6–11.5</t>
         </is>
       </c>
       <c r="F30" s="14" t="n">
@@ -56187,7 +56187,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>8.0–13.4</t>
+          <t>7.8–13.4</t>
         </is>
       </c>
       <c r="H30" s="14" t="n">
@@ -56195,7 +56195,7 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>14.6–21.3</t>
+          <t>14.5–21.4</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
@@ -56203,7 +56203,7 @@
       </c>
       <c r="K30" s="13" t="inlineStr">
         <is>
-          <t>6.9–11.4</t>
+          <t>6.9–11.6</t>
         </is>
       </c>
       <c r="L30" s="14" t="n">
@@ -56211,7 +56211,7 @@
       </c>
       <c r="M30" s="13" t="inlineStr">
         <is>
-          <t>7.7–13.4</t>
+          <t>7.9–13.7</t>
         </is>
       </c>
     </row>
@@ -56226,7 +56226,7 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>2.8–4.8</t>
+          <t>2.8–4.6</t>
         </is>
       </c>
       <c r="D31" s="16" t="n">
@@ -56234,7 +56234,7 @@
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>6.7–9.7</t>
+          <t>6.6–9.5</t>
         </is>
       </c>
       <c r="F31" s="16" t="n">
@@ -56242,7 +56242,7 @@
       </c>
       <c r="G31" s="15" t="inlineStr">
         <is>
-          <t>5.0–6.0</t>
+          <t>5.0–5.9</t>
         </is>
       </c>
       <c r="H31" s="16" t="n">
@@ -56250,7 +56250,7 @@
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
-          <t>2.9–4.7</t>
+          <t>2.8–4.7</t>
         </is>
       </c>
       <c r="J31" s="16" t="n">
@@ -56258,7 +56258,7 @@
       </c>
       <c r="K31" s="15" t="inlineStr">
         <is>
-          <t>6.6–9.6</t>
+          <t>6.7–9.6</t>
         </is>
       </c>
       <c r="L31" s="16" t="n">
@@ -56281,7 +56281,7 @@
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>6.8–9.6</t>
+          <t>6.9–9.3</t>
         </is>
       </c>
       <c r="D32" s="14" t="n">
@@ -56289,7 +56289,7 @@
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>7.4–11.5</t>
+          <t>7.1–12.0</t>
         </is>
       </c>
       <c r="F32" s="14" t="n">
@@ -56297,7 +56297,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>6.4–7.6</t>
+          <t>6.2–7.7</t>
         </is>
       </c>
       <c r="H32" s="14" t="n">
@@ -56305,7 +56305,7 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>4.9–7.2</t>
+          <t>4.8–7.3</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
@@ -56313,7 +56313,7 @@
       </c>
       <c r="K32" s="13" t="inlineStr">
         <is>
-          <t>8.0–12.8</t>
+          <t>8.1–13.4</t>
         </is>
       </c>
       <c r="L32" s="14" t="n">
@@ -56321,7 +56321,7 @@
       </c>
       <c r="M32" s="13" t="inlineStr">
         <is>
-          <t>0.4–1.0</t>
+          <t>0.4–0.9</t>
         </is>
       </c>
     </row>
@@ -56344,7 +56344,7 @@
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>10.3–13.4</t>
+          <t>10.3–13.6</t>
         </is>
       </c>
       <c r="F33" s="16" t="n">
@@ -56360,7 +56360,7 @@
       </c>
       <c r="I33" s="15" t="inlineStr">
         <is>
-          <t>0.8–1.9</t>
+          <t>0.8–2.0</t>
         </is>
       </c>
       <c r="J33" s="16" t="n">
@@ -56368,7 +56368,7 @@
       </c>
       <c r="K33" s="15" t="inlineStr">
         <is>
-          <t>10.7–14.2</t>
+          <t>10.7–14.4</t>
         </is>
       </c>
       <c r="L33" s="16" t="n">
@@ -56391,7 +56391,7 @@
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>20.8–26.4</t>
+          <t>21.1–26.2</t>
         </is>
       </c>
       <c r="D34" s="14" t="n">
@@ -56407,7 +56407,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>18.8–24.0</t>
+          <t>18.4–23.6</t>
         </is>
       </c>
       <c r="H34" s="14" t="n">
@@ -56415,7 +56415,7 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>21.3–26.1</t>
+          <t>21.1–25.9</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
@@ -56423,7 +56423,7 @@
       </c>
       <c r="K34" s="13" t="inlineStr">
         <is>
-          <t>18.6–23.7</t>
+          <t>19.0–23.7</t>
         </is>
       </c>
       <c r="L34" s="14" t="n">
@@ -56431,7 +56431,7 @@
       </c>
       <c r="M34" s="13" t="inlineStr">
         <is>
-          <t>18.6–23.4</t>
+          <t>18.5–23.6</t>
         </is>
       </c>
     </row>
@@ -56446,7 +56446,7 @@
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>0.7–1.9</t>
+          <t>0.8–1.9</t>
         </is>
       </c>
       <c r="D35" s="16" t="n">
@@ -56454,7 +56454,7 @@
       </c>
       <c r="E35" s="15" t="inlineStr">
         <is>
-          <t>4.2–7.7</t>
+          <t>4.1–7.6</t>
         </is>
       </c>
       <c r="F35" s="16" t="n">
@@ -56462,7 +56462,7 @@
       </c>
       <c r="G35" s="15" t="inlineStr">
         <is>
-          <t>6.1–9.4</t>
+          <t>6.1–9.3</t>
         </is>
       </c>
       <c r="H35" s="16" t="n">
@@ -56470,7 +56470,7 @@
       </c>
       <c r="I35" s="15" t="inlineStr">
         <is>
-          <t>0.8–1.9</t>
+          <t>0.7–1.9</t>
         </is>
       </c>
       <c r="J35" s="16" t="n">
@@ -56478,7 +56478,7 @@
       </c>
       <c r="K35" s="15" t="inlineStr">
         <is>
-          <t>4.0–7.6</t>
+          <t>4.1–7.4</t>
         </is>
       </c>
       <c r="L35" s="16" t="n">
@@ -56486,7 +56486,7 @@
       </c>
       <c r="M35" s="15" t="inlineStr">
         <is>
-          <t>5.9–9.5</t>
+          <t>5.8–9.3</t>
         </is>
       </c>
     </row>
@@ -60194,11 +60194,11 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="D27" s="16" t="n">
-        <v>298.32</v>
+        <v>290.63</v>
       </c>
       <c r="E27" s="25" t="n">
         <v>6</v>
@@ -60218,11 +60218,11 @@
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="D28" s="14" t="n">
-        <v>290.63</v>
+        <v>298.32</v>
       </c>
       <c r="E28" s="23" t="n">
         <v>6</v>
@@ -60266,11 +60266,11 @@
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="D30" s="14" t="n">
-        <v>114.75</v>
+        <v>81.04000000000001</v>
       </c>
       <c r="E30" s="23" t="n">
         <v>6</v>
@@ -60290,11 +60290,11 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="D31" s="16" t="n">
-        <v>81.04000000000001</v>
+        <v>114.75</v>
       </c>
       <c r="E31" s="25" t="n">
         <v>6</v>
@@ -60338,11 +60338,11 @@
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="D33" s="16" t="n">
-        <v>240.83</v>
+        <v>174.35</v>
       </c>
       <c r="E33" s="25" t="n">
         <v>6</v>
@@ -60362,11 +60362,11 @@
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="D34" s="14" t="n">
-        <v>174.35</v>
+        <v>240.83</v>
       </c>
       <c r="E34" s="23" t="n">
         <v>6</v>
@@ -60410,11 +60410,11 @@
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="D36" s="14" t="n">
-        <v>286.59</v>
+        <v>286.18</v>
       </c>
       <c r="E36" s="23" t="n">
         <v>6</v>
@@ -60434,11 +60434,11 @@
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="D37" s="16" t="n">
-        <v>286.18</v>
+        <v>286.59</v>
       </c>
       <c r="E37" s="25" t="n">
         <v>6</v>
@@ -60482,11 +60482,11 @@
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="D39" s="16" t="n">
-        <v>157.36</v>
+        <v>97.61</v>
       </c>
       <c r="E39" s="25" t="n">
         <v>6</v>
@@ -60506,11 +60506,11 @@
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="D40" s="14" t="n">
-        <v>97.61</v>
+        <v>157.36</v>
       </c>
       <c r="E40" s="23" t="n">
         <v>6</v>
@@ -60554,11 +60554,11 @@
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="D42" s="14" t="n">
-        <v>149.43</v>
+        <v>298.67</v>
       </c>
       <c r="E42" s="23" t="n">
         <v>6</v>
@@ -60578,11 +60578,11 @@
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="D43" s="16" t="n">
-        <v>298.67</v>
+        <v>149.43</v>
       </c>
       <c r="E43" s="25" t="n">
         <v>6</v>
@@ -62019,7 +62019,7 @@
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -62028,16 +62028,16 @@
         </is>
       </c>
       <c r="D35" s="27" t="n">
-        <v>3860</v>
+        <v>3904</v>
       </c>
       <c r="E35" s="14" t="n">
-        <v>5.65</v>
+        <v>8.31</v>
       </c>
       <c r="F35" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G35" s="24" t="n">
-        <v>0.01744</v>
+        <v>0.00394</v>
       </c>
     </row>
     <row r="36">
@@ -62046,7 +62046,7 @@
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
@@ -62055,10 +62055,10 @@
         </is>
       </c>
       <c r="D36" s="28" t="n">
-        <v>3860</v>
+        <v>3904</v>
       </c>
       <c r="E36" s="16" t="n">
-        <v>75.13</v>
+        <v>34.12</v>
       </c>
       <c r="F36" s="25" t="n">
         <v>5</v>
@@ -62073,7 +62073,7 @@
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -62082,16 +62082,16 @@
         </is>
       </c>
       <c r="D37" s="27" t="n">
-        <v>3904</v>
+        <v>3860</v>
       </c>
       <c r="E37" s="14" t="n">
-        <v>8.31</v>
+        <v>5.65</v>
       </c>
       <c r="F37" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G37" s="24" t="n">
-        <v>0.00394</v>
+        <v>0.01744</v>
       </c>
     </row>
     <row r="38">
@@ -62100,7 +62100,7 @@
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
@@ -62109,10 +62109,10 @@
         </is>
       </c>
       <c r="D38" s="28" t="n">
-        <v>3904</v>
+        <v>3860</v>
       </c>
       <c r="E38" s="16" t="n">
-        <v>34.12</v>
+        <v>75.13</v>
       </c>
       <c r="F38" s="25" t="n">
         <v>5</v>
@@ -62181,7 +62181,7 @@
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -62190,16 +62190,16 @@
         </is>
       </c>
       <c r="D41" s="27" t="n">
-        <v>4035</v>
+        <v>4046</v>
       </c>
       <c r="E41" s="14" t="n">
-        <v>5.46</v>
+        <v>0.38</v>
       </c>
       <c r="F41" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G41" s="24" t="n">
-        <v>0.01951</v>
+        <v>0.53851</v>
       </c>
     </row>
     <row r="42">
@@ -62208,7 +62208,7 @@
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
@@ -62217,16 +62217,16 @@
         </is>
       </c>
       <c r="D42" s="28" t="n">
-        <v>4035</v>
+        <v>4046</v>
       </c>
       <c r="E42" s="16" t="n">
-        <v>94.38</v>
+        <v>10.61</v>
       </c>
       <c r="F42" s="25" t="n">
         <v>5</v>
       </c>
       <c r="G42" s="26" t="n">
-        <v>0</v>
+        <v>0.05964</v>
       </c>
     </row>
     <row r="43">
@@ -62235,7 +62235,7 @@
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -62244,16 +62244,16 @@
         </is>
       </c>
       <c r="D43" s="27" t="n">
-        <v>4046</v>
+        <v>4035</v>
       </c>
       <c r="E43" s="14" t="n">
-        <v>0.38</v>
+        <v>5.46</v>
       </c>
       <c r="F43" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G43" s="24" t="n">
-        <v>0.53851</v>
+        <v>0.01951</v>
       </c>
     </row>
     <row r="44">
@@ -62262,7 +62262,7 @@
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
@@ -62271,16 +62271,16 @@
         </is>
       </c>
       <c r="D44" s="28" t="n">
-        <v>4046</v>
+        <v>4035</v>
       </c>
       <c r="E44" s="16" t="n">
-        <v>10.61</v>
+        <v>94.38</v>
       </c>
       <c r="F44" s="25" t="n">
         <v>5</v>
       </c>
       <c r="G44" s="26" t="n">
-        <v>0.05964</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -62343,7 +62343,7 @@
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -62352,16 +62352,16 @@
         </is>
       </c>
       <c r="D47" s="27" t="n">
-        <v>4804</v>
+        <v>4775</v>
       </c>
       <c r="E47" s="14" t="n">
-        <v>4.68</v>
+        <v>3.92</v>
       </c>
       <c r="F47" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G47" s="24" t="n">
-        <v>0.03044</v>
+        <v>0.04774</v>
       </c>
     </row>
     <row r="48">
@@ -62370,7 +62370,7 @@
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>Wasting (BB/TB)</t>
+          <t>Underweight (BB/U)</t>
         </is>
       </c>
       <c r="C48" s="15" t="inlineStr">
@@ -62379,16 +62379,16 @@
         </is>
       </c>
       <c r="D48" s="28" t="n">
-        <v>4804</v>
+        <v>4775</v>
       </c>
       <c r="E48" s="16" t="n">
-        <v>14.29</v>
+        <v>27.55</v>
       </c>
       <c r="F48" s="25" t="n">
         <v>5</v>
       </c>
       <c r="G48" s="26" t="n">
-        <v>0.01388</v>
+        <v>4e-05</v>
       </c>
     </row>
     <row r="49">
@@ -62397,7 +62397,7 @@
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -62406,16 +62406,16 @@
         </is>
       </c>
       <c r="D49" s="27" t="n">
-        <v>4775</v>
+        <v>4804</v>
       </c>
       <c r="E49" s="14" t="n">
-        <v>3.92</v>
+        <v>4.68</v>
       </c>
       <c r="F49" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G49" s="24" t="n">
-        <v>0.04774</v>
+        <v>0.03044</v>
       </c>
     </row>
     <row r="50">
@@ -62424,7 +62424,7 @@
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>Underweight (BB/U)</t>
+          <t>Wasting (BB/TB)</t>
         </is>
       </c>
       <c r="C50" s="15" t="inlineStr">
@@ -62433,16 +62433,16 @@
         </is>
       </c>
       <c r="D50" s="28" t="n">
-        <v>4775</v>
+        <v>4804</v>
       </c>
       <c r="E50" s="16" t="n">
-        <v>27.55</v>
+        <v>14.29</v>
       </c>
       <c r="F50" s="25" t="n">
         <v>5</v>
       </c>
       <c r="G50" s="26" t="n">
-        <v>4e-05</v>
+        <v>0.01388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>